<commit_message>
Add benchmark matching system with complete benchmarks and test endpoint
</commit_message>
<xml_diff>
--- a/docs/benchmark-objectives-by-kpi-2026-04-10.xlsx
+++ b/docs/benchmark-objectives-by-kpi-2026-04-10.xlsx
@@ -5,12 +5,12 @@
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://enovate92-my.sharepoint.com/personal/jmeyer_e-novate_fr/Documents/Bureau/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://enovate92-my.sharepoint.com/personal/jmeyer_e-novate_fr/Documents/Documents/dev/dev/alerting_enovate/docs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="3" documentId="11_0BA4116F6139B44CC8E53949F9998A2ABFED8057" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{739B5686-9B1D-44DA-BB79-FF52D5D659FF}"/>
+  <xr:revisionPtr revIDLastSave="19" documentId="11_0BA4116F6139B44CC8E53949F9998A2ABFED8057" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6D58ED64-59A2-45C9-9DBA-AEAFE7EEBDE6}"/>
   <bookViews>
-    <workbookView minimized="1" xWindow="10590" yWindow="1455" windowWidth="14400" windowHeight="8310" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="14" activeTab="18" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="CTR" sheetId="1" r:id="rId1"/>
@@ -31,13 +31,14 @@
     <sheet name="Brandsafety" sheetId="16" r:id="rId16"/>
     <sheet name="Reach" sheetId="17" r:id="rId17"/>
     <sheet name="Attention publicitaire" sheetId="18" r:id="rId18"/>
+    <sheet name="JSON Export" sheetId="19" r:id="rId19"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1011" uniqueCount="208">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1014" uniqueCount="211">
   <si>
     <t>Règle</t>
   </si>
@@ -661,16 +662,1367 @@
   </si>
   <si>
     <t>Score d'efficacité</t>
+  </si>
+  <si>
+    <t xml:space="preserve">{
+  "CTR": {
+    "colonnes": [
+      "Règle",
+      "Libellé",
+      "Mesureurs",
+      "Normes IAS",
+      "Catégories d'annonceur",
+      "Annonceurs",
+      "Formats",
+      "Devices",
+      "Types",
+      "Fonctionnalités",
+      "CTR (%)"
+    ],
+    "règles": [
+      {
+        "Règle": 1,
+        "Libellé": "Habillage Desktop",
+        "Mesureurs": "Tous les mesureurs",
+        "Normes IAS": "Toutes les normes",
+        "Catégories d'annonceur": "Toutes les catégories",
+        "Annonceurs": "Tous les annonceurs",
+        "Formats": "Habillage",
+        "Devices": "Desktop",
+        "Types": "Tous les types",
+        "Fonctionnalités": "Toutes les fonctionnalités",
+        "CTR (%)": "0.26 - 0.32"
+      },
+      {
+        "Règle": 2,
+        "Libellé": "Grand Angle",
+        "Mesureurs": "Tous les mesureurs",
+        "Normes IAS": "Toutes les normes",
+        "Catégories d'annonceur": "Toutes les catégories",
+        "Annonceurs": "Tous les annonceurs",
+        "Formats": "Grand Angle",
+        "Devices": "Tous les devices",
+        "Types": "Tous les types",
+        "Fonctionnalités": "Toutes les fonctionnalités",
+        "CTR (%)": "0.26 - 0.33"
+      },
+      {
+        "Règle": 3,
+        "Libellé": "Native",
+        "Mesureurs": "Tous les mesureurs",
+        "Normes IAS": "Toutes les normes",
+        "Catégories d'annonceur": "Toutes les catégories",
+        "Annonceurs": "Tous les annonceurs",
+        "Formats": "Native",
+        "Devices": "Tous les devices",
+        "Types": "Tous les types",
+        "Fonctionnalités": "Toutes les fonctionnalités",
+        "CTR (%)": "0.71 - 0.82"
+      },
+      {
+        "Règle": 4,
+        "Libellé": "Pavé",
+        "Mesureurs": "Tous les mesureurs",
+        "Normes IAS": "Toutes les normes",
+        "Catégories d'annonceur": "Toutes les catégories",
+        "Annonceurs": "Tous les annonceurs",
+        "Formats": "Pavé",
+        "Devices": "Tous les devices",
+        "Types": "Tous les types",
+        "Fonctionnalités": "Toutes les fonctionnalités",
+        "CTR (%)": "0.15 - 0.2"
+      },
+      {
+        "Règle": 5,
+        "Libellé": "Parallaxe Mobile",
+        "Mesureurs": "Tous les mesureurs",
+        "Normes IAS": "Toutes les normes",
+        "Catégories d'annonceur": "Toutes les catégories",
+        "Annonceurs": "Tous les annonceurs",
+        "Formats": "Parallaxe",
+        "Devices": "Mobile",
+        "Types": "Tous les types",
+        "Fonctionnalités": "Toutes les fonctionnalités",
+        "CTR (%)": "0.63 - 0.73"
+      },
+      {
+        "Règle": 6,
+        "Libellé": "Bannière",
+        "Mesureurs": "Tous les mesureurs",
+        "Normes IAS": "Toutes les normes",
+        "Catégories d'annonceur": "Toutes les catégories",
+        "Annonceurs": "Tous les annonceurs",
+        "Formats": "Bannière",
+        "Devices": "Tous les devices",
+        "Types": "Tous les types",
+        "Fonctionnalités": "Toutes les fonctionnalités",
+        "CTR (%)": "0.17 - 0.23"
+      },
+      {
+        "Règle": 7,
+        "Libellé": "Interstitiel Mobile",
+        "Mesureurs": "Tous les mesureurs",
+        "Normes IAS": "Toutes les normes",
+        "Catégories d'annonceur": "Toutes les catégories",
+        "Annonceurs": "Tous les annonceurs",
+        "Formats": "Interstitiel",
+        "Devices": "Mobile",
+        "Types": "Tous les types",
+        "Fonctionnalités": "Toutes les fonctionnalités",
+        "CTR (%)": "4.46 - 4.71"
+      },
+      {
+        "Règle": 8,
+        "Libellé": "Habillage Statique Desktop",
+        "Mesureurs": "Tous les mesureurs",
+        "Normes IAS": "Toutes les normes",
+        "Catégories d'annonceur": "Toutes les catégories",
+        "Annonceurs": "Tous les annonceurs",
+        "Formats": "Habillage",
+        "Devices": "Desktop",
+        "Types": "Statique",
+        "Fonctionnalités": "Toutes les fonctionnalités",
+        "CTR (%)": "0.26 - 0.32"
+      },
+      {
+        "Règle": 9,
+        "Libellé": "Habillage Animé Desktop",
+        "Mesureurs": "Tous les mesureurs",
+        "Normes IAS": "Toutes les normes",
+        "Catégories d'annonceur": "Toutes les catégories",
+        "Annonceurs": "Tous les annonceurs",
+        "Formats": "Habillage",
+        "Devices": "Desktop",
+        "Types": "Animé",
+        "Fonctionnalités": "Toutes les fonctionnalités",
+        "CTR (%)": "0.25 - 0.32"
+      },
+      {
+        "Règle": 10,
+        "Libellé": "Grand Angle Animé Mobile",
+        "Mesureurs": "Tous les mesureurs",
+        "Normes IAS": "Toutes les normes",
+        "Catégories d'annonceur": "Toutes les catégories",
+        "Annonceurs": "Tous les annonceurs",
+        "Formats": "Grand Angle",
+        "Devices": "Mobile",
+        "Types": "Animé",
+        "Fonctionnalités": "Toutes les fonctionnalités",
+        "CTR (%)": "0.32 - 0.39"
+      },
+      {
+        "Règle": 11,
+        "Libellé": "Pavé Animé Mobile",
+        "Mesureurs": "Tous les mesureurs",
+        "Normes IAS": "Toutes les normes",
+        "Catégories d'annonceur": "Toutes les catégories",
+        "Annonceurs": "Tous les annonceurs",
+        "Formats": "Pavé",
+        "Devices": "Mobile",
+        "Types": "Animé",
+        "Fonctionnalités": "Toutes les fonctionnalités",
+        "CTR (%)": "0.13 - 0.18"
+      },
+      {
+        "Règle": 12,
+        "Libellé": "Interstitiel Animé Mobile",
+        "Mesureurs": "Tous les mesureurs",
+        "Normes IAS": "Toutes les normes",
+        "Catégories d'annonceur": "Toutes les catégories",
+        "Annonceurs": "Tous les annonceurs",
+        "Formats": "Interstitiel",
+        "Devices": "Mobile",
+        "Types": "Animé",
+        "Fonctionnalités": "Toutes les fonctionnalités",
+        "CTR (%)": "4.56 - 4.81"
+      },
+      {
+        "Règle": 13,
+        "Libellé": "Bannière Animé Mobile",
+        "Mesureurs": "Tous les mesureurs",
+        "Normes IAS": "Toutes les normes",
+        "Catégories d'annonceur": "Toutes les catégories",
+        "Annonceurs": "Tous les annonceurs",
+        "Formats": "Bannière",
+        "Devices": "Mobile",
+        "Types": "Animé",
+        "Fonctionnalités": "Toutes les fonctionnalités",
+        "CTR (%)": "0.16 - 0.2"
+      },
+      {
+        "Règle": 14,
+        "Libellé": "Grand Angle Animé Mobile",
+        "Mesureurs": "Tous les mesureurs",
+        "Normes IAS": "Toutes les normes",
+        "Catégories d'annonceur": "Toutes les catégories",
+        "Annonceurs": "Tous les annonceurs",
+        "Formats": "Grand Angle",
+        "Devices": "Mobile",
+        "Types": "Vidéo",
+        "Fonctionnalités": "Toutes les fonctionnalités",
+        "CTR (%)": "0.4 - 0.48"
+      },
+      {
+        "Règle": 15,
+        "Libellé": "Grand Angle Statique Mobile",
+        "Mesureurs": "Tous les mesureurs",
+        "Normes IAS": "Toutes les normes",
+        "Catégories d'annonceur": "Toutes les catégories",
+        "Annonceurs": "Tous les annonceurs",
+        "Formats": "Grand Angle",
+        "Devices": "Mobile",
+        "Types": "Statique",
+        "Fonctionnalités": "Toutes les fonctionnalités",
+        "CTR (%)": "0.21 - 0.27"
+      },
+      {
+        "Règle": 16,
+        "Libellé": "Pavé Vidéo Mobile",
+        "Mesureurs": "Tous les mesureurs",
+        "Normes IAS": "Toutes les normes",
+        "Catégories d'annonceur": "Toutes les catégories",
+        "Annonceurs": "Tous les annonceurs",
+        "Formats": "Pavé",
+        "Devices": "Mobile",
+        "Types": "Vidéo",
+        "Fonctionnalités": "Toutes les fonctionnalités",
+        "CTR (%)": "0.14 - 0.19"
+      },
+      {
+        "Règle": 17,
+        "Libellé": "Pavé Statique Mobile",
+        "Mesureurs": "Tous les mesureurs",
+        "Normes IAS": "Toutes les normes",
+        "Catégories d'annonceur": "Toutes les catégories",
+        "Annonceurs": "Tous les annonceurs",
+        "Formats": "Pavé",
+        "Devices": "Mobile",
+        "Types": "Statique",
+        "Fonctionnalités": "Toutes les fonctionnalités",
+        "CTR (%)": "0.16 - 0.21"
+      },
+      {
+        "Règle": 18,
+        "Libellé": "Parallaxe Statique Mobile",
+        "Mesureurs": "Tous les mesureurs",
+        "Normes IAS": "Toutes les normes",
+        "Catégories d'annonceur": "Toutes les catégories",
+        "Annonceurs": "Tous les annonceurs",
+        "Formats": "Parallaxe",
+        "Devices": "Mobile",
+        "Types": "Statique",
+        "Fonctionnalités": "Toutes les fonctionnalités",
+        "CTR (%)": "0.47 - 0.56"
+      },
+      {
+        "Règle": 19,
+        "Libellé": "Bannière Vidéo Mobile",
+        "Mesureurs": "Tous les mesureurs",
+        "Normes IAS": "Toutes les normes",
+        "Catégories d'annonceur": "Toutes les catégories",
+        "Annonceurs": "Tous les annonceurs",
+        "Formats": "Bannière",
+        "Devices": "Mobile",
+        "Types": "Vidéo",
+        "Fonctionnalités": "Toutes les fonctionnalités",
+        "CTR (%)": "0.29 - 0.36"
+      },
+      {
+        "Règle": 20,
+        "Libellé": "Bannière Statique Mobile",
+        "Mesureurs": "Tous les mesureurs",
+        "Normes IAS": "Toutes les normes",
+        "Catégories d'annonceur": "Toutes les catégories",
+        "Annonceurs": "Tous les annonceurs",
+        "Formats": "Bannière",
+        "Devices": "Mobile",
+        "Types": "Statique",
+        "Fonctionnalités": "Toutes les fonctionnalités",
+        "CTR (%)": "0.2 - 0.26"
+      },
+      {
+        "Règle": 21,
+        "Libellé": "Interstitiel Vidéo Mobile",
+        "Mesureurs": "Tous les mesureurs",
+        "Normes IAS": "Toutes les normes",
+        "Catégories d'annonceur": "Toutes les catégories",
+        "Annonceurs": "Tous les annonceurs",
+        "Formats": "Interstitiel",
+        "Devices": "Mobile",
+        "Types": "Vidéo",
+        "Fonctionnalités": "Toutes les fonctionnalités",
+        "CTR (%)": "4.63 - 4.87"
+      },
+      {
+        "Règle": 22,
+        "Libellé": "Interstitiel Statique Mobile",
+        "Mesureurs": "Tous les mesureurs",
+        "Normes IAS": "Toutes les normes",
+        "Catégories d'annonceur": "Toutes les catégories",
+        "Annonceurs": "Tous les annonceurs",
+        "Formats": "Interstitiel",
+        "Devices": "Mobile",
+        "Types": "Statique",
+        "Fonctionnalités": "Toutes les fonctionnalités",
+        "CTR (%)": "4.31 - 4.55"
+      },
+      {
+        "Règle": 23,
+        "Libellé": "Interstitiel Configurateur Mobile",
+        "Mesureurs": "Tous les mesureurs",
+        "Normes IAS": "Toutes les normes",
+        "Catégories d'annonceur": "Toutes les catégories",
+        "Annonceurs": "Tous les annonceurs",
+        "Formats": "Interstitiel",
+        "Devices": "Mobile",
+        "Types": "Tous les types",
+        "Fonctionnalités": "Configurateur",
+        "CTR (%)": "5.5 - 5.75"
+      },
+      {
+        "Règle": 24,
+        "Libellé": "Pavé Gaming Mobile",
+        "Mesureurs": "Tous les mesureurs",
+        "Normes IAS": "Toutes les normes",
+        "Catégories d'annonceur": "Toutes les catégories",
+        "Annonceurs": "Tous les annonceurs",
+        "Formats": "Pavé",
+        "Devices": "Mobile",
+        "Types": "Tous les types",
+        "Fonctionnalités": "Gaming",
+        "CTR (%)": "0.02 - 0.04"
+      },
+      {
+        "Règle": 25,
+        "Libellé": "Interstitiel Gaming Mobile",
+        "Mesureurs": "Tous les mesureurs",
+        "Normes IAS": "Toutes les normes",
+        "Catégories d'annonceur": "Toutes les catégories",
+        "Annonceurs": "Tous les annonceurs",
+        "Formats": "Interstitiel",
+        "Devices": "Mobile",
+        "Types": "Tous les types",
+        "Fonctionnalités": "Gaming",
+        "CTR (%)": "2.39 - 2.58"
+      },
+      {
+        "Règle": 26,
+        "Libellé": "Interstitiel Décompte Mobile",
+        "Mesureurs": "Tous les mesureurs",
+        "Normes IAS": "Toutes les normes",
+        "Catégories d'annonceur": "Toutes les catégories",
+        "Annonceurs": "Tous les annonceurs",
+        "Formats": "Interstitiel",
+        "Devices": "Mobile",
+        "Types": "Tous les types",
+        "Fonctionnalités": "Décompte",
+        "CTR (%)": "4.53 - 4.78"
+      },
+      {
+        "Règle": 27,
+        "Libellé": "Interstitiel Carrousel Mobile",
+        "Mesureurs": "Tous les mesureurs",
+        "Normes IAS": "Toutes les normes",
+        "Catégories d'annonceur": "Toutes les catégories",
+        "Annonceurs": "Tous les annonceurs",
+        "Formats": "Interstitiel",
+        "Devices": "Mobile",
+        "Types": "Tous les types",
+        "Fonctionnalités": "Carrousel",
+        "CTR (%)": "4.71 - 4.96"
+      },
+      {
+        "Règle": 28,
+        "Libellé": "Interstitiel Hotspots Mobile",
+        "Mesureurs": "Tous les mesureurs",
+        "Normes IAS": "Toutes les normes",
+        "Catégories d'annonceur": "Toutes les catégories",
+        "Annonceurs": "Tous les annonceurs",
+        "Formats": "Interstitiel",
+        "Devices": "Mobile",
+        "Types": "Tous les types",
+        "Fonctionnalités": "Hotspots",
+        "CTR (%)": "4.64 - 4.89"
+      },
+      {
+        "Règle": 29,
+        "Libellé": "Interstitiel Demi-Fixe Mobile",
+        "Mesureurs": "Tous les mesureurs",
+        "Normes IAS": "Toutes les normes",
+        "Catégories d'annonceur": "Toutes les catégories",
+        "Annonceurs": "Tous les annonceurs",
+        "Formats": "Interstitiel",
+        "Devices": "Mobile",
+        "Types": "Tous les types",
+        "Fonctionnalités": "Demi-fixe",
+        "CTR (%)": "4.25 - 4.5"
+      },
+      {
+        "Règle": 30,
+        "Libellé": "Pavé 3D Mobile",
+        "Mesureurs": "Tous les mesureurs",
+        "Normes IAS": "Toutes les normes",
+        "Catégories d'annonceur": "Toutes les catégories",
+        "Annonceurs": "Tous les annonceurs",
+        "Formats": "Pavé",
+        "Devices": "Mobile",
+        "Types": "Tous les types",
+        "Fonctionnalités": "3D",
+        "CTR (%)": "0.12 - 0.17"
+      },
+      {
+        "Règle": 31,
+        "Libellé": "Interstitiel 3D Mobile",
+        "Mesureurs": "Tous les mesureurs",
+        "Normes IAS": "Toutes les normes",
+        "Catégories d'annonceur": "Toutes les catégories",
+        "Annonceurs": "Tous les annonceurs",
+        "Formats": "Interstitiel",
+        "Devices": "Mobile",
+        "Types": "Tous les types",
+        "Fonctionnalités": "3D",
+        "CTR (%)": "4.76 - 5.01"
+      },
+      {
+        "Règle": 32,
+        "Libellé": "Pavé Grattable Mobile",
+        "Mesureurs": "Tous les mesureurs",
+        "Normes IAS": "Toutes les normes",
+        "Catégories d'annonceur": "Toutes les catégories",
+        "Annonceurs": "Tous les annonceurs",
+        "Formats": "Pavé",
+        "Devices": "Mobile",
+        "Types": "Tous les types",
+        "Fonctionnalités": "Grattable",
+        "CTR (%)": "0.5 - 0.59"
+      },
+      {
+        "Règle": 33,
+        "Libellé": "Interstitiel Flip Mobile",
+        "Mesureurs": "Tous les mesureurs",
+        "Normes IAS": "Toutes les normes",
+        "Catégories d'annonceur": "Toutes les catégories",
+        "Annonceurs": "Tous les annonceurs",
+        "Formats": "Interstitiel",
+        "Devices": "Mobile",
+        "Types": "Tous les types",
+        "Fonctionnalités": "Flip",
+        "CTR (%)": "2.77 - 2.97"
+      },
+      {
+        "Règle": 34,
+        "Libellé": "Interstitiel Grattable Mobile",
+        "Mesureurs": "Tous les mesureurs",
+        "Normes IAS": "Toutes les normes",
+        "Catégories d'annonceur": "Toutes les catégories",
+        "Annonceurs": "Tous les annonceurs",
+        "Formats": "Interstitiel",
+        "Devices": "Mobile",
+        "Types": "Tous les types",
+        "Fonctionnalités": "Grattable",
+        "CTR (%)": "4.1 - 4.83"
+      },
+      {
+        "Règle": 35,
+        "Libellé": "Interstitiel Drag to Reveal Mobile",
+        "Mesureurs": "Tous les mesureurs",
+        "Normes IAS": "Toutes les normes",
+        "Catégories d'annonceur": "Toutes les catégories",
+        "Annonceurs": "Tous les annonceurs",
+        "Formats": "Interstitiel",
+        "Devices": "Mobile",
+        "Types": "Tous les types",
+        "Fonctionnalités": "Drag to Reveal",
+        "CTR (%)": "3.85 - 4.1"
+      },
+      {
+        "Règle": 36,
+        "Libellé": "Interstitiel Cube Mobile",
+        "Mesureurs": "Tous les mesureurs",
+        "Normes IAS": "Toutes les normes",
+        "Catégories d'annonceur": "Toutes les catégories",
+        "Annonceurs": "Tous les annonceurs",
+        "Formats": "Interstitiel",
+        "Devices": "Mobile",
+        "Types": "Tous les types",
+        "Fonctionnalités": "Cube",
+        "CTR (%)": "4.33 - 4.59"
+      },
+      {
+        "Règle": 37,
+        "Libellé": "Interstitiel Spin 360 Mobile",
+        "Mesureurs": "Tous les mesureurs",
+        "Normes IAS": "Toutes les normes",
+        "Catégories d'annonceur": "Toutes les catégories",
+        "Annonceurs": "Tous les annonceurs",
+        "Formats": "Interstitiel",
+        "Devices": "Mobile",
+        "Types": "Tous les types",
+        "Fonctionnalités": "Spin 360",
+        "CTR (%)": "3.86 - 4.11"
+      }
+    ]
+  },
+  "Complétion vidéo": {
+    "colonnes": [
+      "Règle",
+      "Libellé",
+      "Mesureurs",
+      "Normes IAS",
+      "Catégories d'annonceur",
+      "Annonceurs",
+      "Formats",
+      "Devices",
+      "Types",
+      "Fonctionnalités",
+      "VCR (%)",
+      "Durée (s)"
+    ],
+    "règles": [
+      {
+        "Règle": 1,
+        "Libellé": "Interstitiel 6s-10s Mobile",
+        "Mesureurs": "Tous les mesureurs",
+        "Normes IAS": "Toutes les normes",
+        "Catégories d'annonceur": "Toutes les catégories",
+        "Annonceurs": "Tous les annonceurs",
+        "Formats": "Interstitiel",
+        "Devices": "Tous les devices",
+        "Types": "Tous les types",
+        "Fonctionnalités": "Toutes les fonctionnalités",
+        "VCR (%)": "88.06 - 93.17",
+        "Durée (s)": "6 | 7 | 8 | 9 | 10"
+      },
+      {
+        "Règle": 2,
+        "Libellé": "Interstitiel 11s-15s Mobile",
+        "Mesureurs": "Tous les mesureurs",
+        "Normes IAS": "Toutes les normes",
+        "Catégories d'annonceur": "Toutes les catégories",
+        "Annonceurs": "Tous les annonceurs",
+        "Formats": "Interstitiel",
+        "Devices": "Tous les devices",
+        "Types": "Tous les types",
+        "Fonctionnalités": "Toutes les fonctionnalités",
+        "VCR (%)": "79.18 - 85.84",
+        "Durée (s)": "11 | 12 | 13 | 14 | 15"
+      },
+      {
+        "Règle": 3,
+        "Libellé": "Interstitiel 16s-20s Mobile",
+        "Mesureurs": "Tous les mesureurs",
+        "Normes IAS": "Toutes les normes",
+        "Catégories d'annonceur": "Toutes les catégories",
+        "Annonceurs": "Tous les annonceurs",
+        "Formats": "Interstitiel",
+        "Devices": "Tous les devices",
+        "Types": "Tous les types",
+        "Fonctionnalités": "Toutes les fonctionnalités",
+        "VCR (%)": "71.6 - 79.16",
+        "Durée (s)": "16 | 17 | 18 | 19 | 20"
+      },
+      {
+        "Règle": 4,
+        "Libellé": "Interstitiel 21s-25s Mobile",
+        "Mesureurs": "Tous les mesureurs",
+        "Normes IAS": "Toutes les normes",
+        "Catégories d'annonceur": "Toutes les catégories",
+        "Annonceurs": "Tous les annonceurs",
+        "Formats": "Interstitiel",
+        "Devices": "Tous les devices",
+        "Types": "Tous les types",
+        "Fonctionnalités": "Toutes les fonctionnalités",
+        "VCR (%)": "77.84 - 84.68",
+        "Durée (s)": "21 | 22 | 23 | 24 | 25"
+      },
+      {
+        "Règle": 5,
+        "Libellé": "Interstitiel 26s-30s Mobile",
+        "Mesureurs": "Tous les mesureurs",
+        "Normes IAS": "Toutes les normes",
+        "Catégories d'annonceur": "Toutes les catégories",
+        "Annonceurs": "Tous les annonceurs",
+        "Formats": "Interstitiel",
+        "Devices": "Tous les devices",
+        "Types": "Tous les types",
+        "Fonctionnalités": "Toutes les fonctionnalités",
+        "VCR (%)": "56.26 - 65.79",
+        "Durée (s)": "26 | 27 | 28 | 29 | 30"
+      },
+      {
+        "Règle": 6,
+        "Libellé": "Pavé 6s-10s Mobile",
+        "Mesureurs": "Tous les mesureurs",
+        "Normes IAS": "Toutes les normes",
+        "Catégories d'annonceur": "Toutes les catégories",
+        "Annonceurs": "Tous les annonceurs",
+        "Formats": "Pavé",
+        "Devices": "Tous les devices",
+        "Types": "Tous les types",
+        "Fonctionnalités": "Toutes les fonctionnalités",
+        "VCR (%)": "81.01 - 87.4",
+        "Durée (s)": "6 | 7 | 8 | 9 | 10"
+      },
+      {
+        "Règle": 7,
+        "Libellé": "Pavé 11s-15s Mobile",
+        "Mesureurs": "Tous les mesureurs",
+        "Normes IAS": "Toutes les normes",
+        "Catégories d'annonceur": "Toutes les catégories",
+        "Annonceurs": "Tous les annonceurs",
+        "Formats": "Pavé",
+        "Devices": "Tous les devices",
+        "Types": "Tous les types",
+        "Fonctionnalités": "Toutes les fonctionnalités",
+        "VCR (%)": "72.25 - 79.74",
+        "Durée (s)": "11 | 12 | 13 | 14 | 15"
+      },
+      {
+        "Règle": 8,
+        "Libellé": "Pavé 16s-20s Mobile",
+        "Mesureurs": "Tous les mesureurs",
+        "Normes IAS": "Toutes les normes",
+        "Catégories d'annonceur": "Toutes les catégories",
+        "Annonceurs": "Tous les annonceurs",
+        "Formats": "Pavé",
+        "Devices": "Tous les devices",
+        "Types": "Tous les types",
+        "Fonctionnalités": "Toutes les fonctionnalités",
+        "VCR (%)": "66.14 - 74.16",
+        "Durée (s)": "16 | 17 | 18 | 19 | 20"
+      },
+      {
+        "Règle": 9,
+        "Libellé": "Pavé 21s-25s Mobile",
+        "Mesureurs": "Tous les mesureurs",
+        "Normes IAS": "Toutes les normes",
+        "Catégories d'annonceur": "Toutes les catégories",
+        "Annonceurs": "Tous les annonceurs",
+        "Formats": "Pavé",
+        "Devices": "Tous les devices",
+        "Types": "Tous les types",
+        "Fonctionnalités": "Toutes les fonctionnalités",
+        "VCR (%)": "60.93 - 69.28",
+        "Durée (s)": "21 | 22 | 23 | 24 | 25"
+      },
+      {
+        "Règle": 10,
+        "Libellé": "Pavé 26s-30s Mobile",
+        "Mesureurs": "Tous les mesureurs",
+        "Normes IAS": "Toutes les normes",
+        "Catégories d'annonceur": "Toutes les catégories",
+        "Annonceurs": "Tous les annonceurs",
+        "Formats": "Pavé",
+        "Devices": "Tous les devices",
+        "Types": "Tous les types",
+        "Fonctionnalités": "Toutes les fonctionnalités",
+        "VCR (%)": "9.5 - 15.28",
+        "Durée (s)": "26 | 27 | 28 | 29 | 30"
+      },
+      {
+        "Règle": 11,
+        "Libellé": "Pré-roll 11s-15s Mobile",
+        "Mesureurs": "Tous les mesureurs",
+        "Normes IAS": "Toutes les normes",
+        "Catégories d'annonceur": "Toutes les catégories",
+        "Annonceurs": "Tous les annonceurs",
+        "Formats": "Pré-roll",
+        "Devices": "Tous les devices",
+        "Types": "Tous les types",
+        "Fonctionnalités": "Toutes les fonctionnalités",
+        "VCR (%)": "81.14 - 87.51",
+        "Durée (s)": "11 | 12 | 13 | 14 | 15"
+      },
+      {
+        "Règle": 12,
+        "Libellé": "Pré-roll 16s-20s Mobile",
+        "Mesureurs": "Tous les mesureurs",
+        "Normes IAS": "Toutes les normes",
+        "Catégories d'annonceur": "Toutes les catégories",
+        "Annonceurs": "Tous les annonceurs",
+        "Formats": "Pré-roll",
+        "Devices": "Tous les devices",
+        "Types": "Tous les types",
+        "Fonctionnalités": "Toutes les fonctionnalités",
+        "VCR (%)": "87.83 - 92.99",
+        "Durée (s)": "16 | 17 | 18 | 19 | 20"
+      },
+      {
+        "Règle": 13,
+        "Libellé": "Pré-roll 21s-25s Mobile",
+        "Mesureurs": "Tous les mesureurs",
+        "Normes IAS": "Toutes les normes",
+        "Catégories d'annonceur": "Toutes les catégories",
+        "Annonceurs": "Tous les annonceurs",
+        "Formats": "Pré-roll",
+        "Devices": "Tous les devices",
+        "Types": "Tous les types",
+        "Fonctionnalités": "Toutes les fonctionnalités",
+        "VCR (%)": "65.69 - 73.75",
+        "Durée (s)": "21 | 22 | 23 | 24 | 25"
+      },
+      {
+        "Règle": 14,
+        "Libellé": "Pré-roll 26s-30s Mobile",
+        "Mesureurs": "Tous les mesureurs",
+        "Normes IAS": "Toutes les normes",
+        "Catégories d'annonceur": "Toutes les catégories",
+        "Annonceurs": "Tous les annonceurs",
+        "Formats": "Pré-roll",
+        "Devices": "Tous les devices",
+        "Types": "Tous les types",
+        "Fonctionnalités": "Toutes les fonctionnalités",
+        "VCR (%)": "49.07 - 57.82",
+        "Durée (s)": "26 | 27 | 28 | 29 | 30"
+      },
+      {
+        "Règle": 15,
+        "Libellé": "Grand Angle 21s-25s Mobile",
+        "Mesureurs": "Tous les mesureurs",
+        "Normes IAS": "Toutes les normes",
+        "Catégories d'annonceur": "Toutes les catégories",
+        "Annonceurs": "Tous les annonceurs",
+        "Formats": "Grand Angle",
+        "Devices": "Tous les devices",
+        "Types": "Tous les types",
+        "Fonctionnalités": "Toutes les fonctionnalités",
+        "VCR (%)": "41.08 - 49.81",
+        "Durée (s)": "21 | 22 | 23 | 24 | 25"
+      }
+    ]
+  },
+  "Visibilité": {
+    "colonnes": [
+      "Règle",
+      "Libellé",
+      "Mesureurs",
+      "Normes IAS",
+      "Catégories d'annonceur",
+      "Annonceurs",
+      "Formats",
+      "Devices",
+      "Types",
+      "Fonctionnalités",
+      "Taux de visibilité (%)"
+    ],
+    "règles": [
+      {
+        "Règle": 1,
+        "Libellé": "Pré-roll Mobile",
+        "Mesureurs": "Tous les mesureurs",
+        "Normes IAS": "Toutes les normes",
+        "Catégories d'annonceur": "Toutes les catégories",
+        "Annonceurs": "Tous les annonceurs",
+        "Formats": "Pré-roll",
+        "Devices": "Mobile",
+        "Types": "Tous les types",
+        "Fonctionnalités": "Toutes les fonctionnalités",
+        "Taux de visibilité (%)": null
+      },
+      {
+        "Règle": 2,
+        "Libellé": "Grand Angle Mobile",
+        "Mesureurs": "Tous les mesureurs",
+        "Normes IAS": "Toutes les normes",
+        "Catégories d'annonceur": "Toutes les catégories",
+        "Annonceurs": "Tous les annonceurs",
+        "Formats": "Grand Angle",
+        "Devices": "Mobile",
+        "Types": "Tous les types",
+        "Fonctionnalités": "Toutes les fonctionnalités",
+        "Taux de visibilité (%)": null
+      },
+      {
+        "Règle": 3,
+        "Libellé": "Pavé Mobile",
+        "Mesureurs": "Tous les mesureurs",
+        "Normes IAS": "Toutes les normes",
+        "Catégories d'annonceur": "Toutes les catégories",
+        "Annonceurs": "Tous les annonceurs",
+        "Formats": "Pavé",
+        "Devices": "Mobile",
+        "Types": "Tous les types",
+        "Fonctionnalités": "Toutes les fonctionnalités",
+        "Taux de visibilité (%)": null
+      },
+      {
+        "Règle": 4,
+        "Libellé": "Bannière Mobile",
+        "Mesureurs": "Tous les mesureurs",
+        "Normes IAS": "Toutes les normes",
+        "Catégories d'annonceur": "Toutes les catégories",
+        "Annonceurs": "Tous les annonceurs",
+        "Formats": "Bannière",
+        "Devices": "Mobile",
+        "Types": "Tous les types",
+        "Fonctionnalités": "Toutes les fonctionnalités",
+        "Taux de visibilité (%)": null
+      },
+      {
+        "Règle": 5,
+        "Libellé": "Interstitiel Mobile",
+        "Mesureurs": "Tous les mesureurs",
+        "Normes IAS": "Toutes les normes",
+        "Catégories d'annonceur": "Toutes les catégories",
+        "Annonceurs": "Tous les annonceurs",
+        "Formats": "Interstitiel",
+        "Devices": "Mobile",
+        "Types": "Tous les types",
+        "Fonctionnalités": "Toutes les fonctionnalités",
+        "Taux de visibilité (%)": null
+      }
+    ]
+  },
+  "Taux de visite LP": {
+    "colonnes": [
+      "Règle",
+      "Libellé",
+      "Mesureurs",
+      "Normes IAS",
+      "Catégories d'annonceur",
+      "Annonceurs",
+      "Formats",
+      "Devices",
+      "Types",
+      "Fonctionnalités",
+      "Taux de visite LP (%)",
+      "Taux d'interaction LP (%)"
+    ],
+    "règles": [
+      {
+        "Règle": 1,
+        "Libellé": "Bannière Mobile",
+        "Mesureurs": "Tous les mesureurs",
+        "Normes IAS": "Toutes les normes",
+        "Catégories d'annonceur": "Toutes les catégories",
+        "Annonceurs": "Tous les annonceurs",
+        "Formats": "Bannière",
+        "Devices": "Mobile",
+        "Types": "Tous les types",
+        "Fonctionnalités": "Toutes les fonctionnalités",
+        "Taux de visite LP (%)": "60.76 - 66.72",
+        "Taux d'interaction LP (%)": "1.78 - 3.82"
+      },
+      {
+        "Règle": 2,
+        "Libellé": "Pavé Mobile",
+        "Mesureurs": "Tous les mesureurs",
+        "Normes IAS": "Toutes les normes",
+        "Catégories d'annonceur": "Toutes les catégories",
+        "Annonceurs": "Tous les annonceurs",
+        "Formats": "Pavé",
+        "Devices": "Mobile",
+        "Types": "Tous les types",
+        "Fonctionnalités": "Toutes les fonctionnalités",
+        "Taux de visite LP (%)": "53.77 - 59.91",
+        "Taux d'interaction LP (%)": "1.84 - 3.9"
+      },
+      {
+        "Règle": 3,
+        "Libellé": "Interstitiel Mobile",
+        "Mesureurs": "Tous les mesureurs",
+        "Normes IAS": "Toutes les normes",
+        "Catégories d'annonceur": "Toutes les catégories",
+        "Annonceurs": "Tous les annonceurs",
+        "Formats": "Interstitiel",
+        "Devices": "Mobile",
+        "Types": "Tous les types",
+        "Fonctionnalités": "Toutes les fonctionnalités",
+        "Taux de visite LP (%)": "63.05 - 68.93",
+        "Taux d'interaction LP (%)": "5.91 - 9.19"
+      },
+      {
+        "Règle": 4,
+        "Libellé": "Global",
+        "Mesureurs": "Tous les mesureurs",
+        "Normes IAS": "Toutes les normes",
+        "Catégories d'annonceur": "Toutes les catégories",
+        "Annonceurs": "Tous les annonceurs",
+        "Formats": "Tous les formats",
+        "Devices": "Mobile",
+        "Types": "Tous les types",
+        "Fonctionnalités": "Toutes les fonctionnalités",
+        "Taux de visite LP (%)": "63.25 - 69.11",
+        "Taux d'interaction LP (%)": "5.68 - 8.91"
+      }
+    ]
+  },
+  "Taux de session": {
+    "colonnes": [
+      "Règle",
+      "Libellé",
+      "Mesureurs",
+      "Normes IAS",
+      "Catégories d'annonceur",
+      "Annonceurs",
+      "Formats",
+      "Devices",
+      "Types",
+      "Fonctionnalités",
+      "Taux de session",
+      "CPV"
+    ],
+    "règles": []
+  },
+  "Taux de session conditionné": {
+    "colonnes": [
+      "Règle",
+      "Libellé",
+      "Mesureurs",
+      "Normes IAS",
+      "Catégories d'annonceur",
+      "Annonceurs",
+      "Formats",
+      "Devices",
+      "Types",
+      "Fonctionnalités",
+      "Taux de session conditionné",
+      "CPV"
+    ],
+    "règles": []
+  },
+  "Taux de Rebond Temps passé": {
+    "colonnes": [
+      "Règle",
+      "Libellé",
+      "Mesureurs",
+      "Normes IAS",
+      "Catégories d'annonceur",
+      "Annonceurs",
+      "Formats",
+      "Devices",
+      "Types",
+      "Fonctionnalités",
+      "Taux de session",
+      "Taux de rebond",
+      "Temps passé moyen"
+    ],
+    "règles": [
+      {
+        "Règle": 1,
+        "Libellé": null,
+        "Mesureurs": "Tous les mesureurs",
+        "Normes IAS": "Toutes les normes",
+        "Catégories d'annonceur": "Toutes les catégories",
+        "Annonceurs": "Tous les annonceurs",
+        "Formats": "Tous les formats",
+        "Devices": "Tous les devices",
+        "Types": "Tous les types",
+        "Fonctionnalités": "Toutes les fonctionnalités",
+        "Taux de session": null,
+        "Taux de rebond": null,
+        "Temps passé moyen": null
+      }
+    ]
+  },
+  "Taux de Rebond Temps passé Cond": {
+    "colonnes": [
+      "Règle",
+      "Libellé",
+      "Mesureurs",
+      "Normes IAS",
+      "Catégories d'annonceur",
+      "Annonceurs",
+      "Formats",
+      "Devices",
+      "Types",
+      "Fonctionnalités",
+      "Taux de session conditionné",
+      "Taux de rebond",
+      "Temps passé moyen"
+    ],
+    "règles": []
+  },
+  "Taux de Rebond Nombre de pages ": {
+    "colonnes": [
+      "Règle",
+      "Libellé",
+      "Mesureurs",
+      "Normes IAS",
+      "Catégories d'annonceur",
+     </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> "Annonceurs",
+      "Formats",
+      "Devices",
+      "Types",
+      "Fonctionnalités",
+      "Taux de session",
+      "Taux de rebond",
+      "Temps passé moyen",
+      "Nombre de pages vues"
+    ],
+    "règles": []
+  },
+  "Taux de Rebond Nombre de page 2": {
+    "colonnes": [
+      "Règle",
+      "Libellé",
+      "Mesureurs",
+      "Normes IAS",
+      "Catégories d'annonceur",
+      "Annonceurs",
+      "Formats",
+      "Devices",
+      "Types",
+      "Fonctionnalités",
+      "Taux de session conditionné",
+      "Taux de rebond",
+      "Temps passé moyen",
+      "Nombre de pages vues"
+    ],
+    "règles": []
+  },
+  "Visites en Magasin CTR": {
+    "colonnes": [
+      "Règle",
+      "Libellé",
+      "Mesureurs",
+      "Normes IAS",
+      "Catégories d'annonceur",
+      "Annonceurs",
+      "Formats",
+      "Devices",
+      "Types",
+      "Fonctionnalités",
+      "CPVI",
+      "CTR"
+    ],
+    "règles": []
+  },
+  "Visites en Magasin Taux de Visi": {
+    "colonnes": [
+      "Règle",
+      "Libellé",
+      "Mesureurs",
+      "Normes IAS",
+      "Catégories d'annonceur",
+      "Annonceurs",
+      "Formats",
+      "Devices",
+      "Types",
+      "Fonctionnalités",
+      "CPVI",
+      "Taux de visite LP",
+      "Taux d'interaction LP"
+    ],
+    "règles": []
+  },
+  "Leads": {
+    "colonnes": [
+      "Règle",
+      "Libellé",
+      "Mesureurs",
+      "Normes IAS",
+      "Catégories d'annonceur",
+      "Annonceurs",
+      "Formats",
+      "Devices",
+      "Types",
+      "Fonctionnalités",
+      "CPL (€)",
+      "Leads"
+    ],
+    "règles": []
+  },
+  "Couverture sur Cible (DAR)": {
+    "colonnes": [
+      "Règle",
+      "Libellé",
+      "Mesureurs",
+      "Normes IAS",
+      "Catégories d'annonceur",
+      "Annonceurs",
+      "Formats",
+      "Devices",
+      "Types",
+      "Fonctionnalités",
+      "Taux d'interaction format (%)"
+    ],
+    "règles": []
+  },
+  "Interaction Format": {
+    "colonnes": [
+      "Règle",
+      "Libellé",
+      "Mesureurs",
+      "Normes IAS",
+      "Catégories d'annonceur",
+      "Annonceurs",
+      "Formats",
+      "Devices",
+      "Types",
+      "Fonctionnalités",
+      "Taux d'interaction format (%)"
+    ],
+    "règles": [
+      {
+        "Règle": 1,
+        "Libellé": "Interstitiel Configurateur Moble",
+        "Mesureurs": "Tous les mesureurs",
+        "Normes IAS": "Toutes les normes",
+        "Catégories d'annonceur": "Toutes les catégories",
+        "Annonceurs": "Tous les annonceurs",
+        "Formats": "Interstitiel",
+        "Devices": "Mobile",
+        "Types": "Tous les types",
+        "Fonctionnalités": "Configurateur",
+        "Taux d'interaction format (%)": "4.04 - 4.86"
+      },
+      {
+        "Règle": 2,
+        "Libellé": "Interstitiel Gaming Mobile",
+        "Mesureurs": "Tous les mesureurs",
+        "Normes IAS": "Toutes les normes",
+        "Catégories d'annonceur": "Toutes les catégories",
+        "Annonceurs": "Tous les annonceurs",
+        "Formats": "Interstitiel",
+        "Devices": "Mobile",
+        "Types": "Tous les types",
+        "Fonctionnalités": "Gaming",
+        "Taux d'interaction format (%)": "3.46 - 3.77"
+      },
+      {
+        "Règle": 3,
+        "Libellé": "Pavé Carrousel Mobile",
+        "Mesureurs": "Tous les mesureurs",
+        "Normes IAS": "Toutes les normes",
+        "Catégories d'annonceur": "Toutes les catégories",
+        "Annonceurs": "Tous les annonceurs",
+        "Formats": "Pavé",
+        "Devices": "Mobile",
+        "Types": "Tous les types",
+        "Fonctionnalités": "Carrousel",
+        "Taux d'interaction format (%)": "3.64 - 4.41"
+      },
+      {
+        "Règle": 4,
+        "Libellé": "Interstitiel Carrousel Mobile",
+        "Mesureurs": "Tous les mesureurs",
+        "Normes IAS": "Toutes les normes",
+        "Catégories d'annonceur": "Toutes les catégories",
+        "Annonceurs": "Tous les annonceurs",
+        "Formats": "Interstitiel",
+        "Devices": "Mobile",
+        "Types": "Tous les types",
+        "Fonctionnalités": "Carrousel",
+        "Taux d'interaction format (%)": "4.12 - 4.94"
+      },
+      {
+        "Règle": 5,
+        "Libellé": "Interstitiel 3D Mobile",
+        "Mesureurs": "Tous les mesureurs",
+        "Normes IAS": "Toutes les normes",
+        "Catégories d'annonceur": "Toutes les catégories",
+        "Annonceurs": "Tous les annonceurs",
+        "Formats": "Interstitiel",
+        "Devices": "Mobile",
+        "Types": "Tous les types",
+        "Fonctionnalités": "3D",
+        "Taux d'interaction format (%)": "1.84 - 2.41"
+      },
+      {
+        "Règle": 6,
+        "Libellé": "Grand Angle Flip Mobile",
+        "Mesureurs": "Tous les mesureurs",
+        "Normes IAS": "Toutes les normes",
+        "Catégories d'annonceur": "Toutes les catégories",
+        "Annonceurs": "Tous les annonceurs",
+        "Formats": "Grand Angle",
+        "Devices": "Mobile",
+        "Types": "Tous les types",
+        "Fonctionnalités": "Flip",
+        "Taux d'interaction format (%)": "3.11 - 3.82"
+      }
+    ]
+  },
+  "Brandsafety": {
+    "colonnes": [
+      "Règle",
+      "Libellé",
+      "Mesureurs",
+      "Normes IAS",
+      "Catégories d'annonceur",
+      "Annonceurs",
+      "Formats",
+      "Devices",
+      "Types",
+      "Fonctionnalités",
+      "Taux de Brandsafety",
+      "Taux de Brandsuitability",
+      "Taux d'Invalid Trafic"
+    ],
+    "règles": [
+      {
+        "Règle": 1,
+        "Libellé": "Native",
+        "Mesureurs": "Tous les mesureurs",
+        "Normes IAS": "Toutes les normes",
+        "Catégories d'annonceur": "Toutes les catégories",
+        "Annonceurs": "Tous les annonceurs",
+        "Formats": "Native",
+        "Devices": "Tous les devices",
+        "Types": "Tous les types",
+        "Fonctionnalités": "Toutes les fonctionnalités",
+        "Taux de Brandsafety": "97.87 - 98.05",
+        "Taux de Brandsuitability": null,
+        "Taux d'Invalid Trafic": null
+      },
+      {
+        "Règle": 2,
+        "Libellé": "Pré-roll",
+        "Mesureurs": "Tous les mesureurs",
+        "Normes IAS": "Toutes les normes",
+        "Catégories d'annonceur": "Toutes les catégories",
+        "Annonceurs": "Tous les annonceurs",
+        "Formats": "Pré-roll",
+        "Devices": "Tous les devices",
+        "Types": "Tous les types",
+        "Fonctionnalités": "Toutes les fonctionnalités",
+        "Taux de Brandsafety": "97.86 - 98.04",
+        "Taux de Brandsuitability": null,
+        "Taux d'Invalid Trafic": null
+      },
+      {
+        "Règle": 3,
+        "Libellé": "Grand Angle",
+        "Mesureurs": "Tous les mesureurs",
+        "Normes IAS": "Toutes les normes",
+        "Catégories d'annonceur": "Toutes les catégories",
+        "Annonceurs": "Tous les annonceurs",
+        "Formats": "Grand Angle",
+        "Devices": "Tous les devices",
+        "Types": "Tous les types",
+        "Fonctionnalités": "Toutes les fonctionnalités",
+        "Taux de Brandsafety": "99.76 - 99.82",
+        "Taux de Brandsuitability": null,
+        "Taux d'Invalid Trafic": null
+      },
+      {
+        "Règle": 4,
+        "Libellé": "Pavé",
+        "Mesureurs": "Tous les mesureurs",
+        "Normes IAS": "Toutes les normes",
+        "Catégories d'annonceur": "Toutes les catégories",
+        "Annonceurs": "Tous les annonceurs",
+        "Formats": "Pavé",
+        "Devices": "Tous les devices",
+        "Types": "Tous les types",
+        "Fonctionnalités": "Toutes les fonctionnalités",
+        "Taux de Brandsafety": "99.63 - 99.71",
+        "Taux de Brandsuitability": null,
+        "Taux d'Invalid Trafic": null
+      },
+      {
+        "Règle": 5,
+        "Libellé": "Parallaxe",
+        "Mesureurs": "Tous les mesureurs",
+        "Normes IAS": "Toutes les normes",
+        "Catégories d'annonceur": "Toutes les catégories",
+        "Annonceurs": "Tous les annonceurs",
+        "Formats": "Parallaxe",
+        "Devices": "Tous les devices",
+        "Types": "Tous les types",
+        "Fonctionnalités": "Toutes les fonctionnalités",
+        "Taux de Brandsafety": "97.82 - 97.99",
+        "Taux de Brandsuitability": null,
+        "Taux d'Invalid Trafic": null
+      },
+      {
+        "Règle": 6,
+        "Libellé": "Bannière",
+        "Mesureurs": "Tous les mesureurs",
+        "Normes IAS": "Toutes les normes",
+        "Catégories d'annonceur": "Toutes les catégories",
+        "Annonceurs": "Tous les annonceurs",
+        "Formats": "Bannière",
+        "Devices": "Tous les devices",
+        "Types": "Tous les types",
+        "Fonctionnalités": "Toutes les fonctionnalités",
+        "Taux de Brandsafety": "99.61 - 99.68",
+        "Taux de Brandsuitability": null,
+        "Taux d'Invalid Trafic": null
+      },
+      {
+        "Règle": 7,
+        "Libellé": "Interstitiel",
+        "Mesureurs": "Tous les mesureurs",
+        "Normes IAS": "Toutes les normes",
+        "Catégories d'annonceur": "Toutes les catégories",
+        "Annonceurs": "Tous les annonceurs",
+        "Formats": "Interstitiel",
+        "Devices": "Tous les devices",
+        "Types": "Tous les types",
+        "Fonctionnalités": "Toutes les fonctionnalités",
+        "Taux de Brandsafety": "99.35 - 99.44",
+        "Taux de Brandsuitability": null,
+        "Taux d'Invalid Trafic": null
+      }
+    ]
+  },
+  "Reach": {
+    "colonnes": [
+      "Règle",
+      "Libellé",
+      "Mesureurs",
+      "Normes IAS",
+      "Catégories d'annonceur",
+      "Annonceurs",
+      "Formats",
+      "Devices",
+      "Types",
+      "Fonctionnalités",
+      "Capping de répétition"
+    ],
+    "règles": []
+  },
+  "Attention publicitaire": {
+    "colonnes": [
+      "Règle",
+      "Libellé",
+      "Mesureurs",
+      "Normes IAS",
+      "Catégories d'annonceur",
+      "Annonceurs",
+      "Formats",
+      "Devices",
+      "Types",
+      "Fonctionnalités",
+      "Temps d'attention moyen (s)",
+      "Taux d'attention (%)",
+      "Taux d'attention 1s (%)",
+      "Taux d'attention 2s (%)",
+      "Taux d'attention 3s (%)",
+      "Taux d'attention 4s (%)",
+      "Taux d'attention 5s (%)",
+      "Score d'attention",
+      "Score d'efficacité"
+    ],
+    "règles": []
+  }
+}</t>
+  </si>
+  <si>
+    <t>← Le JSON est dans A1 et A2 (concaténez les deux)</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="12"/>
+      <color rgb="FF666666"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -696,8 +2048,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1035,17 +2392,39 @@
 </a:theme>
 </file>
 
+<file path=xl/webextensions/taskpanes.xml><?xml version="1.0" encoding="utf-8"?>
+<wetp:taskpanes xmlns:wetp="http://schemas.microsoft.com/office/webextensions/taskpanes/2010/11">
+  <wetp:taskpane dockstate="right" visibility="0" width="350" row="5">
+    <wetp:webextensionref xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </wetp:taskpane>
+</wetp:taskpanes>
+</file>
+
+<file path=xl/webextensions/webextension1.xml><?xml version="1.0" encoding="utf-8"?>
+<we:webextension xmlns:we="http://schemas.microsoft.com/office/webextensions/webextension/2010/11" id="{95CE6950-5E0D-4D59-912B-3F20DFCEDD5C}">
+  <we:reference id="WA200009404" version="1.0.0.8" store="Omex" storeType="OMEX"/>
+  <we:alternateReferences>
+    <we:reference id="WA200009404" version="1.0.0.8" store="WA200009404" storeType="OMEX"/>
+  </we:alternateReferences>
+  <we:properties>
+    <we:property name="claude.fileId" value="&quot;b065b27e-1b0a-4006-bc42-ee3e64a7ad66&quot;"/>
+  </we:properties>
+  <we:bindings/>
+  <we:snapshot xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships"/>
+</we:webextension>
+</file>
+
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:K38"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="28.25" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="16.75" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="15.75" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1080,7 +2459,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="2" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>1</v>
       </c>
@@ -1115,7 +2494,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="3" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>2</v>
       </c>
@@ -1150,7 +2529,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="4" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>3</v>
       </c>
@@ -1185,7 +2564,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="5" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>4</v>
       </c>
@@ -1220,7 +2599,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="6" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>5</v>
       </c>
@@ -1255,7 +2634,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="7" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>6</v>
       </c>
@@ -1290,7 +2669,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="8" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>7</v>
       </c>
@@ -1325,7 +2704,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="9" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>8</v>
       </c>
@@ -1360,7 +2739,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="10" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>9</v>
       </c>
@@ -1395,7 +2774,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="11" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>10</v>
       </c>
@@ -1430,7 +2809,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="12" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>11</v>
       </c>
@@ -1465,7 +2844,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="13" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>12</v>
       </c>
@@ -1500,7 +2879,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="14" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>13</v>
       </c>
@@ -1535,7 +2914,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="15" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A15">
         <v>14</v>
       </c>
@@ -1570,7 +2949,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="16" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A16">
         <v>15</v>
       </c>
@@ -1605,7 +2984,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="17" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A17">
         <v>16</v>
       </c>
@@ -1640,7 +3019,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="18" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A18">
         <v>17</v>
       </c>
@@ -1675,7 +3054,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="19" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A19">
         <v>18</v>
       </c>
@@ -1710,7 +3089,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="20" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A20">
         <v>19</v>
       </c>
@@ -1745,7 +3124,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="21" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A21">
         <v>20</v>
       </c>
@@ -1780,7 +3159,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="22" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A22">
         <v>21</v>
       </c>
@@ -1815,7 +3194,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="23" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A23">
         <v>22</v>
       </c>
@@ -1850,7 +3229,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="24" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A24">
         <v>23</v>
       </c>
@@ -1885,7 +3264,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="25" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A25">
         <v>24</v>
       </c>
@@ -1920,7 +3299,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="26" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A26">
         <v>25</v>
       </c>
@@ -1955,7 +3334,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="27" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A27">
         <v>26</v>
       </c>
@@ -1990,7 +3369,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="28" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A28">
         <v>27</v>
       </c>
@@ -2025,7 +3404,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="29" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A29">
         <v>28</v>
       </c>
@@ -2060,7 +3439,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="30" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A30">
         <v>29</v>
       </c>
@@ -2095,7 +3474,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="31" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A31">
         <v>30</v>
       </c>
@@ -2130,7 +3509,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="32" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A32">
         <v>31</v>
       </c>
@@ -2165,7 +3544,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="33" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A33">
         <v>32</v>
       </c>
@@ -2200,7 +3579,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="34" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A34">
         <v>33</v>
       </c>
@@ -2235,7 +3614,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="35" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A35">
         <v>34</v>
       </c>
@@ -2270,7 +3649,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="36" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A36">
         <v>35</v>
       </c>
@@ -2305,7 +3684,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="37" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A37">
         <v>36</v>
       </c>
@@ -2340,7 +3719,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="38" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A38">
         <v>37</v>
       </c>
@@ -2386,9 +3765,9 @@
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0900-000000000000}">
   <dimension ref="A1:N1"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:14" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -2443,9 +3822,9 @@
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0A00-000000000000}">
   <dimension ref="A1:L1"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:12" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -2494,9 +3873,9 @@
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0B00-000000000000}">
   <dimension ref="A1:M1"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -2548,9 +3927,9 @@
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0C00-000000000000}">
   <dimension ref="A1:L1"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:12" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -2599,9 +3978,9 @@
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0D00-000000000000}">
   <dimension ref="A1:K1"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -2647,9 +4026,9 @@
 <file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0E00-000000000000}">
   <dimension ref="A1:K7"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -2684,7 +4063,7 @@
         <v>178</v>
       </c>
     </row>
-    <row r="2" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>1</v>
       </c>
@@ -2719,7 +4098,7 @@
         <v>180</v>
       </c>
     </row>
-    <row r="3" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>2</v>
       </c>
@@ -2754,7 +4133,7 @@
         <v>181</v>
       </c>
     </row>
-    <row r="4" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>3</v>
       </c>
@@ -2789,7 +4168,7 @@
         <v>183</v>
       </c>
     </row>
-    <row r="5" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>4</v>
       </c>
@@ -2824,7 +4203,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="6" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>5</v>
       </c>
@@ -2859,7 +4238,7 @@
         <v>185</v>
       </c>
     </row>
-    <row r="7" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>6</v>
       </c>
@@ -2905,9 +4284,9 @@
 <file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0F00-000000000000}">
   <dimension ref="A1:M8"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -2948,7 +4327,7 @@
         <v>190</v>
       </c>
     </row>
-    <row r="2" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>1</v>
       </c>
@@ -2989,7 +4368,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="3" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>2</v>
       </c>
@@ -3030,7 +4409,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="4" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>3</v>
       </c>
@@ -3071,7 +4450,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="5" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>4</v>
       </c>
@@ -3112,7 +4491,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="6" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>5</v>
       </c>
@@ -3153,7 +4532,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="7" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>6</v>
       </c>
@@ -3194,7 +4573,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="8" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>7</v>
       </c>
@@ -3246,9 +4625,9 @@
 <file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1000-000000000000}">
   <dimension ref="A1:K1"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -3294,9 +4673,9 @@
 <file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1100-000000000000}">
   <dimension ref="A1:S1"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:19" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -3363,12 +4742,39 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{94CCF462-E5BD-4139-AEC4-01C65EAC9354}">
+  <dimension ref="A1:B2"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="100" style="2" customWidth="1"/>
+    <col min="2" max="2" width="66.625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A1" s="3" t="s">
+        <v>208</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A2" s="3" t="s">
+        <v>209</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:L16"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:12" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -3406,7 +4812,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="2" spans="1:12" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>1</v>
       </c>
@@ -3444,7 +4850,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="3" spans="1:12" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>2</v>
       </c>
@@ -3482,7 +4888,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="4" spans="1:12" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>3</v>
       </c>
@@ -3520,7 +4926,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="5" spans="1:12" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>4</v>
       </c>
@@ -3558,7 +4964,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="6" spans="1:12" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>5</v>
       </c>
@@ -3596,7 +5002,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="7" spans="1:12" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>6</v>
       </c>
@@ -3634,7 +5040,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="8" spans="1:12" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>7</v>
       </c>
@@ -3672,7 +5078,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="9" spans="1:12" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>8</v>
       </c>
@@ -3710,7 +5116,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="10" spans="1:12" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>9</v>
       </c>
@@ -3748,7 +5154,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="11" spans="1:12" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>10</v>
       </c>
@@ -3786,7 +5192,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="12" spans="1:12" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>11</v>
       </c>
@@ -3824,7 +5230,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="13" spans="1:12" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>12</v>
       </c>
@@ -3862,7 +5268,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="14" spans="1:12" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>13</v>
       </c>
@@ -3900,7 +5306,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="15" spans="1:12" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A15">
         <v>14</v>
       </c>
@@ -3938,7 +5344,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="16" spans="1:12" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A16">
         <v>15</v>
       </c>
@@ -3987,9 +5393,9 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:K6"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -4024,7 +5430,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="2" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>1</v>
       </c>
@@ -4059,7 +5465,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="3" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>2</v>
       </c>
@@ -4094,7 +5500,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="4" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>3</v>
       </c>
@@ -4129,7 +5535,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="5" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>4</v>
       </c>
@@ -4164,7 +5570,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="6" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>5</v>
       </c>
@@ -4210,9 +5616,9 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:L5"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:12" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -4250,7 +5656,7 @@
         <v>155</v>
       </c>
     </row>
-    <row r="2" spans="1:12" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>1</v>
       </c>
@@ -4288,7 +5694,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="3" spans="1:12" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>2</v>
       </c>
@@ -4326,7 +5732,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="4" spans="1:12" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>3</v>
       </c>
@@ -4364,7 +5770,7 @@
         <v>161</v>
       </c>
     </row>
-    <row r="5" spans="1:12" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>4</v>
       </c>
@@ -4413,9 +5819,9 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:L1"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:12" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -4464,9 +5870,9 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <dimension ref="A1:L1"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:12" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -4515,9 +5921,9 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
   <dimension ref="A1:M2"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -4558,7 +5964,7 @@
         <v>170</v>
       </c>
     </row>
-    <row r="2" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>1</v>
       </c>
@@ -4610,9 +6016,9 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
   <dimension ref="A1:M1"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -4664,9 +6070,9 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0800-000000000000}">
   <dimension ref="A1:N1"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:14" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>

</xml_diff>